<commit_message>
Some analysis performed, missing pairwise comparison, models
</commit_message>
<xml_diff>
--- a/raw_data/Fines_study.xlsx
+++ b/raw_data/Fines_study.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yacordob\Documents\GitHub\Fines_Study\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F75127B-0607-4DE6-B32A-87C265413778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE2364B-FBA1-432D-8D94-53E7B0CCA0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6774BC92-58FD-4C69-B304-20496453BFDA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{6774BC92-58FD-4C69-B304-20496453BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="Pulping" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="280">
   <si>
     <t>Biomass</t>
   </si>
@@ -878,6 +878,12 @@
   </si>
   <si>
     <t>ID1</t>
+  </si>
+  <si>
+    <t>E1AN4</t>
+  </si>
+  <si>
+    <t>E1AN1</t>
   </si>
 </sst>
 </file>
@@ -950,7 +956,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -971,14 +977,13 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2646,21 +2651,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
       <c r="H1" s="5"/>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
     </row>
     <row r="2" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
@@ -5650,7 +5655,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="B13">
         <v>1.3226</v>
@@ -5804,7 +5809,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>159</v>
+        <v>278</v>
       </c>
       <c r="B24">
         <v>1.3011999999999999</v>
@@ -5818,7 +5823,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>140</v>
+        <v>279</v>
       </c>
       <c r="B25">
         <v>1.2509999999999999</v>
@@ -7482,357 +7487,356 @@
     <col min="2" max="2" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" t="s">
         <v>273</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" t="s">
         <v>277</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" t="s">
         <v>275</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" t="s">
         <v>276</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="18" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" t="s">
         <v>271</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="18">
+      <c r="D2">
         <v>500</v>
       </c>
-      <c r="E2" s="18">
+      <c r="E2">
         <v>28</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2">
         <v>2.9670000000000001</v>
       </c>
-      <c r="G2" s="19">
-        <f>F2/1000</f>
+      <c r="G2" s="16">
+        <f t="shared" ref="G2:G13" si="0">F2/1000</f>
         <v>2.967E-3</v>
       </c>
-      <c r="H2" s="18">
+      <c r="H2">
         <v>445</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" t="s">
         <v>272</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="18">
+      <c r="D3">
         <v>600</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3">
         <v>29</v>
       </c>
-      <c r="F3" s="18">
+      <c r="F3">
         <v>2.97</v>
       </c>
-      <c r="G3" s="19">
-        <f>F3/1000</f>
+      <c r="G3" s="16">
+        <f t="shared" si="0"/>
         <v>2.97E-3</v>
       </c>
-      <c r="H3" s="18">
+      <c r="H3">
         <v>554</v>
       </c>
     </row>
-    <row r="4" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="18" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" t="s">
         <v>271</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" t="s">
         <v>108</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4">
         <v>510</v>
       </c>
-      <c r="E4" s="18">
+      <c r="E4">
         <v>28</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4">
         <v>3.08</v>
       </c>
-      <c r="G4" s="19">
-        <f>F4/1000</f>
+      <c r="G4" s="16">
+        <f t="shared" si="0"/>
         <v>3.0800000000000003E-3</v>
       </c>
-      <c r="H4" s="18">
+      <c r="H4">
         <v>464</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" t="s">
         <v>272</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5">
         <v>620</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5">
         <v>30</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5">
         <v>2.7669999999999999</v>
       </c>
-      <c r="G5" s="19">
-        <f>F5/1000</f>
+      <c r="G5" s="16">
+        <f t="shared" si="0"/>
         <v>2.7669999999999999E-3</v>
       </c>
-      <c r="H5" s="18">
+      <c r="H5">
         <v>561</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" t="s">
         <v>271</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6">
         <v>500</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6">
         <v>28</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6">
         <v>3.0670000000000002</v>
       </c>
-      <c r="G6" s="19">
-        <f>F6/1000</f>
+      <c r="G6" s="16">
+        <f t="shared" si="0"/>
         <v>3.0670000000000003E-3</v>
       </c>
-      <c r="H6" s="18">
+      <c r="H6">
         <v>453</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="18" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" t="s">
         <v>272</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" t="s">
         <v>112</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7">
         <v>600</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7">
         <v>29</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7">
         <v>2.9940000000000002</v>
       </c>
-      <c r="G7" s="19">
-        <f>F7/1000</f>
+      <c r="G7" s="16">
+        <f t="shared" si="0"/>
         <v>2.9940000000000001E-3</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7">
         <v>554</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="18" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" t="s">
         <v>271</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" t="s">
         <v>113</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8">
         <v>600</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8">
         <v>28</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8">
         <v>3.0939999999999999</v>
       </c>
-      <c r="G8" s="19">
-        <f>F8/1000</f>
+      <c r="G8" s="16">
+        <f t="shared" si="0"/>
         <v>3.094E-3</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8">
         <v>564</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="18" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" t="s">
         <v>272</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" t="s">
         <v>116</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9">
         <v>670</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9">
         <v>30</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9">
         <v>2.8719999999999999</v>
       </c>
-      <c r="G9" s="19">
-        <f>F9/1000</f>
+      <c r="G9" s="16">
+        <f t="shared" si="0"/>
         <v>2.872E-3</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9">
         <v>628</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" t="s">
         <v>271</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" t="s">
         <v>114</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10">
         <v>610</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10">
         <v>30</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10">
         <v>3.0750000000000002</v>
       </c>
-      <c r="G10" s="19">
-        <f>F10/1000</f>
+      <c r="G10" s="16">
+        <f t="shared" si="0"/>
         <v>3.075E-3</v>
       </c>
-      <c r="H10" s="18">
+      <c r="H10">
         <v>569</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="18" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" t="s">
         <v>272</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" t="s">
         <v>117</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11">
         <v>690</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11">
         <v>31</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11">
         <v>2.706</v>
       </c>
-      <c r="G11" s="19">
-        <f>F11/1000</f>
+      <c r="G11" s="16">
+        <f t="shared" si="0"/>
         <v>2.7060000000000001E-3</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11">
         <v>647</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="18" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" t="s">
         <v>271</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" t="s">
         <v>115</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12">
         <v>630</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12">
         <v>30</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12">
         <v>3.1429999999999998</v>
       </c>
-      <c r="G12" s="19">
-        <f>F12/1000</f>
+      <c r="G12" s="16">
+        <f t="shared" si="0"/>
         <v>3.143E-3</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12">
         <v>599</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="18" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" t="s">
         <v>272</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" t="s">
         <v>118</v>
       </c>
-      <c r="D13" s="18">
+      <c r="D13">
         <v>685</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13">
         <v>30</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13">
         <v>2.8050000000000002</v>
       </c>
-      <c r="G13" s="19">
-        <f>F13/1000</f>
+      <c r="G13" s="16">
+        <f t="shared" si="0"/>
         <v>2.8050000000000002E-3</v>
       </c>
-      <c r="H13" s="18">
+      <c r="H13">
         <v>645</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="14"/>
     </row>

</xml_diff>

<commit_message>
Need to check the column tear is not being saved in line189 code chunk
</commit_message>
<xml_diff>
--- a/raw_data/Fines_study.xlsx
+++ b/raw_data/Fines_study.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yacordob\Documents\GitHub\Fines_Study\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE2364B-FBA1-432D-8D94-53E7B0CCA0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F486A432-9C0D-42E7-836D-253161A735BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{6774BC92-58FD-4C69-B304-20496453BFDA}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="281">
   <si>
     <t>Biomass</t>
   </si>
@@ -884,6 +884,9 @@
   </si>
   <si>
     <t>E1AN1</t>
+  </si>
+  <si>
+    <t>tear_gf</t>
   </si>
 </sst>
 </file>
@@ -5482,10 +5485,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36E2995E-BE9A-41EC-AF23-4F027DDBD2C8}">
-  <dimension ref="A1:D142"/>
+  <dimension ref="A1:E142"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>261</v>
       </c>
@@ -5498,8 +5501,11 @@
       <c r="D1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>138</v>
       </c>
@@ -5513,7 +5519,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>139</v>
       </c>
@@ -5526,8 +5532,11 @@
       <c r="D3" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>140</v>
       </c>
@@ -5540,8 +5549,11 @@
       <c r="D4" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>141</v>
       </c>
@@ -5554,8 +5566,11 @@
       <c r="D5" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E5">
+        <v>17.666666666666668</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>142</v>
       </c>
@@ -5568,8 +5583,11 @@
       <c r="D6" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E6">
+        <v>17.666666666666668</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>143</v>
       </c>
@@ -5582,8 +5600,11 @@
       <c r="D7" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>144</v>
       </c>
@@ -5596,8 +5617,11 @@
       <c r="D8" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>145</v>
       </c>
@@ -5610,8 +5634,11 @@
       <c r="D9" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9">
+        <v>18.333333333333332</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>146</v>
       </c>
@@ -5624,8 +5651,11 @@
       <c r="D10" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10">
+        <v>18.666666666666668</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>147</v>
       </c>
@@ -5639,7 +5669,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>148</v>
       </c>
@@ -5652,8 +5682,11 @@
       <c r="D12" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E12">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>159</v>
       </c>
@@ -5667,7 +5700,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>150</v>
       </c>
@@ -5680,8 +5713,11 @@
       <c r="D14" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E14">
+        <v>17.666666666666668</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>151</v>
       </c>
@@ -5695,7 +5731,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>152</v>
       </c>
@@ -5708,8 +5744,11 @@
       <c r="D16" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E16">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>153</v>
       </c>
@@ -5722,8 +5761,11 @@
       <c r="D17" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>154</v>
       </c>
@@ -5736,8 +5778,11 @@
       <c r="D18" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E18">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>155</v>
       </c>
@@ -5750,8 +5795,11 @@
       <c r="D19" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E19">
+        <v>21.333333333333332</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>156</v>
       </c>
@@ -5765,7 +5813,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>157</v>
       </c>
@@ -5778,8 +5826,11 @@
       <c r="D21" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>149</v>
       </c>
@@ -5792,8 +5843,11 @@
       <c r="D22" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E22">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>158</v>
       </c>
@@ -5807,7 +5861,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>278</v>
       </c>
@@ -5820,8 +5874,11 @@
       <c r="D24" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E24">
+        <v>18.333333333333332</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>279</v>
       </c>
@@ -5835,7 +5892,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>160</v>
       </c>
@@ -5848,8 +5905,11 @@
       <c r="D26" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E26">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>161</v>
       </c>
@@ -5862,8 +5922,11 @@
       <c r="D27" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E27">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>162</v>
       </c>
@@ -5876,8 +5939,11 @@
       <c r="D28" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E28">
+        <v>13.333333333333334</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>163</v>
       </c>
@@ -5891,7 +5957,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>164</v>
       </c>
@@ -5904,8 +5970,11 @@
       <c r="D30" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E30">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>165</v>
       </c>
@@ -5919,7 +5988,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>166</v>
       </c>
@@ -5932,8 +6001,11 @@
       <c r="D32" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E32">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>167</v>
       </c>
@@ -5946,8 +6018,11 @@
       <c r="D33" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E33">
+        <v>11.666666666666666</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>168</v>
       </c>
@@ -5960,8 +6035,11 @@
       <c r="D34" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E34">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>169</v>
       </c>
@@ -5974,8 +6052,11 @@
       <c r="D35" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>170</v>
       </c>
@@ -5989,7 +6070,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>171</v>
       </c>
@@ -6002,8 +6083,11 @@
       <c r="D37" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E37">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>172</v>
       </c>
@@ -6016,8 +6100,11 @@
       <c r="D38" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E38">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>173</v>
       </c>
@@ -6031,7 +6118,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>174</v>
       </c>
@@ -6044,8 +6131,11 @@
       <c r="D40" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E40">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>175</v>
       </c>
@@ -6058,8 +6148,11 @@
       <c r="D41" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E41">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>176</v>
       </c>
@@ -6073,7 +6166,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>177</v>
       </c>
@@ -6086,8 +6179,11 @@
       <c r="D43" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E43">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>178</v>
       </c>
@@ -6100,8 +6196,11 @@
       <c r="D44" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E44">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>179</v>
       </c>
@@ -6114,8 +6213,11 @@
       <c r="D45" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E45">
+        <v>15.333333333333334</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>180</v>
       </c>
@@ -6128,8 +6230,11 @@
       <c r="D46" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E46">
+        <v>17.333333333333332</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>181</v>
       </c>
@@ -6143,7 +6248,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>182</v>
       </c>
@@ -6156,8 +6261,11 @@
       <c r="D48" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E48">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>183</v>
       </c>
@@ -6170,8 +6278,11 @@
       <c r="D49" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E49">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>184</v>
       </c>
@@ -6184,8 +6295,11 @@
       <c r="D50" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E50">
+        <v>24.666666666666668</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>185</v>
       </c>
@@ -6198,8 +6312,11 @@
       <c r="D51" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E51">
+        <v>23.333333333333332</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>186</v>
       </c>
@@ -6212,8 +6329,11 @@
       <c r="D52" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E52">
+        <v>24.666666666666668</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>187</v>
       </c>
@@ -6227,7 +6347,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>188</v>
       </c>
@@ -6240,8 +6360,11 @@
       <c r="D54" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E54">
+        <v>24.666666666666668</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>189</v>
       </c>
@@ -6254,8 +6377,11 @@
       <c r="D55" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E55">
+        <v>24.666666666666668</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>190</v>
       </c>
@@ -6268,8 +6394,11 @@
       <c r="D56" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E56">
+        <v>23.333333333333332</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>191</v>
       </c>
@@ -6283,7 +6412,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>192</v>
       </c>
@@ -6296,8 +6425,11 @@
       <c r="D58" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E58">
+        <v>24.666666666666668</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>193</v>
       </c>
@@ -6310,8 +6442,11 @@
       <c r="D59" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E59">
+        <v>24.666666666666668</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>194</v>
       </c>
@@ -6325,7 +6460,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>195</v>
       </c>
@@ -6338,8 +6473,11 @@
       <c r="D61" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E61">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>196</v>
       </c>
@@ -6353,7 +6491,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>197</v>
       </c>
@@ -6366,8 +6504,11 @@
       <c r="D63" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E63">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>198</v>
       </c>
@@ -6380,8 +6521,11 @@
       <c r="D64" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E64">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>199</v>
       </c>
@@ -6394,8 +6538,11 @@
       <c r="D65" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E65">
+        <v>22.666666666666668</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>200</v>
       </c>
@@ -6409,7 +6556,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>201</v>
       </c>
@@ -6422,8 +6569,11 @@
       <c r="D67" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E67">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>202</v>
       </c>
@@ -6436,8 +6586,11 @@
       <c r="D68" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E68">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>203</v>
       </c>
@@ -6450,8 +6603,11 @@
       <c r="D69" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E69">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>204</v>
       </c>
@@ -6464,8 +6620,11 @@
       <c r="D70" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E70">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>205</v>
       </c>
@@ -6478,8 +6637,11 @@
       <c r="D71" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E71">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>206</v>
       </c>
@@ -6492,8 +6654,11 @@
       <c r="D72" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E72">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>207</v>
       </c>
@@ -6507,7 +6672,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>208</v>
       </c>
@@ -6520,8 +6685,11 @@
       <c r="D74" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E74">
+        <v>24.666666666666668</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>208</v>
       </c>
@@ -6535,7 +6703,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>209</v>
       </c>
@@ -6548,8 +6716,11 @@
       <c r="D76" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E76">
+        <v>25.333333333333332</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>210</v>
       </c>
@@ -6562,8 +6733,11 @@
       <c r="D77" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E77">
+        <v>25.333333333333332</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>211</v>
       </c>
@@ -6577,7 +6751,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>212</v>
       </c>
@@ -6590,8 +6764,11 @@
       <c r="D79" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E79">
+        <v>25.666666666666668</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>213</v>
       </c>
@@ -6604,8 +6781,11 @@
       <c r="D80" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E80">
+        <v>24.666666666666668</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>214</v>
       </c>
@@ -6618,8 +6798,11 @@
       <c r="D81" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E81">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>215</v>
       </c>
@@ -6633,7 +6816,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>216</v>
       </c>
@@ -6647,7 +6830,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>217</v>
       </c>
@@ -6660,8 +6843,11 @@
       <c r="D84" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E84">
+        <v>22.666666666666668</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>218</v>
       </c>
@@ -6674,8 +6860,11 @@
       <c r="D85" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E85">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>219</v>
       </c>
@@ -6688,8 +6877,11 @@
       <c r="D86" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E86">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>220</v>
       </c>
@@ -6702,8 +6894,11 @@
       <c r="D87" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E87">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>221</v>
       </c>
@@ -6717,7 +6912,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>222</v>
       </c>
@@ -6730,8 +6925,11 @@
       <c r="D89" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E89">
+        <v>23.333333333333332</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>223</v>
       </c>
@@ -6744,8 +6942,11 @@
       <c r="D90" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E90">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>224</v>
       </c>
@@ -6759,7 +6960,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>225</v>
       </c>
@@ -6772,8 +6973,11 @@
       <c r="D92" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E92">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>226</v>
       </c>
@@ -6786,8 +6990,11 @@
       <c r="D93" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E93">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>227</v>
       </c>
@@ -6800,8 +7007,11 @@
       <c r="D94" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E94">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>228</v>
       </c>
@@ -6814,8 +7024,11 @@
       <c r="D95" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E95">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>229</v>
       </c>
@@ -6828,8 +7041,11 @@
       <c r="D96" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E96">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>230</v>
       </c>
@@ -6843,7 +7059,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>231</v>
       </c>
@@ -6856,8 +7072,11 @@
       <c r="D98" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E98">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>232</v>
       </c>
@@ -6870,8 +7089,11 @@
       <c r="D99" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E99">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>233</v>
       </c>
@@ -6884,8 +7106,11 @@
       <c r="D100" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E100">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>234</v>
       </c>
@@ -6898,8 +7123,11 @@
       <c r="D101" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E101">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>235</v>
       </c>
@@ -6913,7 +7141,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>236</v>
       </c>
@@ -6926,8 +7154,11 @@
       <c r="D103" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E103">
+        <v>22.666666666666668</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>237</v>
       </c>
@@ -6941,7 +7172,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>238</v>
       </c>
@@ -6954,8 +7185,11 @@
       <c r="D105" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E105">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>239</v>
       </c>
@@ -6968,8 +7202,11 @@
       <c r="D106" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E106">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>119</v>
       </c>
@@ -6982,8 +7219,11 @@
       <c r="D107" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E107">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>122</v>
       </c>
@@ -6997,7 +7237,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>124</v>
       </c>
@@ -7010,8 +7250,11 @@
       <c r="D109" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E109">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>126</v>
       </c>
@@ -7024,8 +7267,11 @@
       <c r="D110" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E110">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>128</v>
       </c>
@@ -7039,7 +7285,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>134</v>
       </c>
@@ -7052,8 +7298,11 @@
       <c r="D112" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E112">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>130</v>
       </c>
@@ -7066,8 +7315,11 @@
       <c r="D113" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E113">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>132</v>
       </c>
@@ -7080,8 +7332,11 @@
       <c r="D114" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E114">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>240</v>
       </c>
@@ -7094,8 +7349,11 @@
       <c r="D115" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E115">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>241</v>
       </c>
@@ -7109,7 +7367,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>242</v>
       </c>
@@ -7122,8 +7380,11 @@
       <c r="D117" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E117">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>243</v>
       </c>
@@ -7136,8 +7397,11 @@
       <c r="D118" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E118">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>244</v>
       </c>
@@ -7150,8 +7414,11 @@
       <c r="D119" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E119">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>245</v>
       </c>
@@ -7165,7 +7432,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>246</v>
       </c>
@@ -7178,8 +7445,11 @@
       <c r="D121" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E121">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>247</v>
       </c>
@@ -7192,8 +7462,11 @@
       <c r="D122" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E122">
+        <v>22.666666666666668</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>248</v>
       </c>
@@ -7206,8 +7479,11 @@
       <c r="D123" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E123">
+        <v>23.333333333333332</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>249</v>
       </c>
@@ -7220,8 +7496,11 @@
       <c r="D124" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E124">
+        <v>21.666666666666668</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>250</v>
       </c>
@@ -7234,8 +7513,11 @@
       <c r="D125" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E125">
+        <v>22.666666666666668</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>251</v>
       </c>
@@ -7249,7 +7531,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>252</v>
       </c>
@@ -7263,7 +7545,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>253</v>
       </c>
@@ -7276,8 +7558,11 @@
       <c r="D128" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E128">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>254</v>
       </c>
@@ -7290,8 +7575,11 @@
       <c r="D129" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E129">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>255</v>
       </c>
@@ -7304,8 +7592,11 @@
       <c r="D130" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E130">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>127</v>
       </c>
@@ -7319,7 +7610,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>123</v>
       </c>
@@ -7332,8 +7623,11 @@
       <c r="D132" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E132">
+        <v>18.666666666666668</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>121</v>
       </c>
@@ -7346,8 +7640,11 @@
       <c r="D133" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E133">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>125</v>
       </c>
@@ -7360,8 +7657,11 @@
       <c r="D134" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E134">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>133</v>
       </c>
@@ -7374,8 +7674,11 @@
       <c r="D135" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E135">
+        <v>22.666666666666668</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>135</v>
       </c>
@@ -7388,8 +7691,11 @@
       <c r="D136" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E136">
+        <v>22.666666666666668</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>129</v>
       </c>
@@ -7403,7 +7709,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>131</v>
       </c>
@@ -7416,8 +7722,11 @@
       <c r="D138" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E138">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>256</v>
       </c>
@@ -7431,7 +7740,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>257</v>
       </c>
@@ -7444,8 +7753,11 @@
       <c r="D140" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E140">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>258</v>
       </c>
@@ -7458,8 +7770,11 @@
       <c r="D141" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E141">
+        <v>20.666666666666668</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>259</v>
       </c>
@@ -7471,6 +7786,9 @@
       </c>
       <c r="D142" t="s">
         <v>120</v>
+      </c>
+      <c r="E142">
+        <v>20.666666666666668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>